<commit_message>
fix privacy governance email escalation flow
</commit_message>
<xml_diff>
--- a/backend/data/privacy_governance_tracker.xlsx
+++ b/backend/data/privacy_governance_tracker.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Privacy Governance Cases'!$A$1:$O$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Approval Evidence'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Approval Evidence'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Governance Dashboard'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -180,7 +180,24 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PrivacyGovernanceDashboardTable" displayName="PrivacyGovernanceDashboardTable" ref="A1:B7" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PrivacyApprovalEvidenceTable" displayName="PrivacyApprovalEvidenceTable" ref="A1:H2" headerRowCount="1">
+  <autoFilter ref="A1:H2"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Approval ID"/>
+    <tableColumn id="2" name="Case ID"/>
+    <tableColumn id="3" name="Change ID"/>
+    <tableColumn id="4" name="Reviewer"/>
+    <tableColumn id="5" name="Role"/>
+    <tableColumn id="6" name="Decision"/>
+    <tableColumn id="7" name="Comment"/>
+    <tableColumn id="8" name="Decided At"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PrivacyGovernanceDashboardTable" displayName="PrivacyGovernanceDashboardTable" ref="A1:B7" headerRowCount="1">
   <autoFilter ref="A1:B7"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Metric"/>
@@ -592,22 +609,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CASE-E2E-003</t>
+          <t>CASE-API-6G-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PCR-E2E-001</t>
+          <t>PCR-API-6G-001</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>New learner data processing</t>
+          <t>6G API decision test</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Beta demonstration of a new privacy-impacting learner processing activity.</t>
+          <t>API decision integration test.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -632,7 +649,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>PENDING_DPO_GRC</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -641,10 +658,16 @@
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>46257.84746179327</v>
-      </c>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
+        <v>46258.8033072658</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>REQUEST_CHANGES</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>46258.80330742644</v>
+      </c>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
     </row>
@@ -663,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -725,9 +748,52 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>APR-GRC-6G-004</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CASE-API-6G-001</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>PCR-API-6G-001</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>GRC Reviewer</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>GRC</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>REQUEST_CHANGES</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>GRC reviewed the case.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>46258.80330742644</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:H2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -786,7 +852,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -806,7 +872,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -816,7 +882,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -826,7 +892,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>46257.84796296297</v>
+        <v>46258.80329861111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete developer admin security and transaction authorization
</commit_message>
<xml_diff>
--- a/backend/data/privacy_governance_tracker.xlsx
+++ b/backend/data/privacy_governance_tracker.xlsx
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>46258.8033072658</v>
+        <v>46275.69055271771</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="M2" s="3" t="n">
-        <v>46258.80330742644</v>
+        <v>46275.69055290536</v>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="H2" s="3" t="n">
-        <v>46258.80330742644</v>
+        <v>46275.69055290536</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>46258.80329861111</v>
+        <v>46275.69054398148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>